<commit_message>
feat: enhance master import with full biodata and add bulk photo zip import by nis
</commit_message>
<xml_diff>
--- a/public/template_import_master.xlsx
+++ b/public/template_import_master.xlsx
@@ -7,7 +7,7 @@
     <workbookView activeTab="0" autoFilterDateGrouping="true" firstSheet="0" minimized="false" showHorizontalScroll="true" showSheetTabs="true" showVerticalScroll="true" tabRatio="600" visibility="visible"/>
   </bookViews>
   <sheets>
-    <sheet name="Worksheet" sheetId="1" r:id="rId4"/>
+    <sheet name="Template Import Master" sheetId="1" r:id="rId4"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="999999" calcMode="auto" calcCompleted="1" fullCalcOnLoad="0" forceFullCalc="0"/>
@@ -15,7 +15,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" uniqueCount="25">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" uniqueCount="83">
   <si>
     <t>nis</t>
   </si>
@@ -26,6 +26,9 @@
     <t>nama</t>
   </si>
   <si>
+    <t>jenis_kelamin</t>
+  </si>
+  <si>
     <t>kode_jurusan</t>
   </si>
   <si>
@@ -38,12 +41,84 @@
     <t>nama_kelas</t>
   </si>
   <si>
+    <t>tmpt_lahir</t>
+  </si>
+  <si>
+    <t>tgl_lahir</t>
+  </si>
+  <si>
+    <t>agama</t>
+  </si>
+  <si>
+    <t>no_hp</t>
+  </si>
+  <si>
+    <t>email</t>
+  </si>
+  <si>
+    <t>alamat</t>
+  </si>
+  <si>
+    <t>rt</t>
+  </si>
+  <si>
+    <t>rw</t>
+  </si>
+  <si>
+    <t>kel</t>
+  </si>
+  <si>
+    <t>kec</t>
+  </si>
+  <si>
+    <t>kota</t>
+  </si>
+  <si>
+    <t>prov</t>
+  </si>
+  <si>
+    <t>no_hp_ibu</t>
+  </si>
+  <si>
+    <t>nama_ibu</t>
+  </si>
+  <si>
+    <t>nik_ibu</t>
+  </si>
+  <si>
+    <t>pekerjaan_ibu</t>
+  </si>
+  <si>
+    <t>no_hp_ayah</t>
+  </si>
+  <si>
+    <t>nama_ayah</t>
+  </si>
+  <si>
+    <t>nik_ayah</t>
+  </si>
+  <si>
+    <t>pekerjaan_ayah</t>
+  </si>
+  <si>
+    <t>no_hp_wali</t>
+  </si>
+  <si>
+    <t>nama_wali</t>
+  </si>
+  <si>
+    <t>233001</t>
+  </si>
+  <si>
     <t>0081234567</t>
   </si>
   <si>
     <t>ANDI WIJAYA</t>
   </si>
   <si>
+    <t>L</t>
+  </si>
+  <si>
     <t>TJKT</t>
   </si>
   <si>
@@ -53,43 +128,142 @@
     <t>X</t>
   </si>
   <si>
-    <t>X-TJKT</t>
+    <t>X-TJKT-1</t>
+  </si>
+  <si>
+    <t>Bandung</t>
+  </si>
+  <si>
+    <t>2008-05-12</t>
+  </si>
+  <si>
+    <t>Islam</t>
+  </si>
+  <si>
+    <t>081234567890</t>
+  </si>
+  <si>
+    <t>andi.wijaya@gmail.com</t>
+  </si>
+  <si>
+    <t>Jl. Merdeka No. 10</t>
+  </si>
+  <si>
+    <t>01</t>
+  </si>
+  <si>
+    <t>03</t>
+  </si>
+  <si>
+    <t>Cihapit</t>
+  </si>
+  <si>
+    <t>Bandung Wetan</t>
+  </si>
+  <si>
+    <t>Kota Bandung</t>
+  </si>
+  <si>
+    <t>Jawa Barat</t>
+  </si>
+  <si>
+    <t>081298765432</t>
+  </si>
+  <si>
+    <t>Siti Rahmah</t>
+  </si>
+  <si>
+    <t>3273015501800001</t>
+  </si>
+  <si>
+    <t>Wiraswasta</t>
+  </si>
+  <si>
+    <t>081211223344</t>
+  </si>
+  <si>
+    <t>Budi Wijaya</t>
+  </si>
+  <si>
+    <t>3273011205780002</t>
+  </si>
+  <si>
+    <t>Karyawan Swasta</t>
+  </si>
+  <si>
+    <t>-</t>
+  </si>
+  <si>
+    <t>233002</t>
   </si>
   <si>
     <t>0087654321</t>
   </si>
   <si>
-    <t>BUDI SANTOSO</t>
-  </si>
-  <si>
-    <t>RPL</t>
-  </si>
-  <si>
-    <t>Rekayasa Perangkat Lunak</t>
-  </si>
-  <si>
-    <t>XI</t>
-  </si>
-  <si>
-    <t>XI-RPL</t>
-  </si>
-  <si>
-    <t>0081122334</t>
-  </si>
-  <si>
-    <t>CITRA DEWI</t>
-  </si>
-  <si>
-    <t>PH</t>
-  </si>
-  <si>
-    <t>Perhotelan</t>
-  </si>
-  <si>
-    <t>XII</t>
-  </si>
-  <si>
-    <t>XII-PH</t>
+    <t>SITI NURHALIZA</t>
+  </si>
+  <si>
+    <t>P</t>
+  </si>
+  <si>
+    <t>MPLB</t>
+  </si>
+  <si>
+    <t>Manajemen Perkantoran dan Layanan Bisnis</t>
+  </si>
+  <si>
+    <t>X-MPLB-1</t>
+  </si>
+  <si>
+    <t>Cimahi</t>
+  </si>
+  <si>
+    <t>2008-08-20</t>
+  </si>
+  <si>
+    <t>081322334455</t>
+  </si>
+  <si>
+    <t>siti.nur@gmail.com</t>
+  </si>
+  <si>
+    <t>Jl. Pasirkaliki No. 45</t>
+  </si>
+  <si>
+    <t>02</t>
+  </si>
+  <si>
+    <t>05</t>
+  </si>
+  <si>
+    <t>Pamoyanan</t>
+  </si>
+  <si>
+    <t>Cicendo</t>
+  </si>
+  <si>
+    <t>081377889900</t>
+  </si>
+  <si>
+    <t>Dewi Sartika</t>
+  </si>
+  <si>
+    <t>3273024508820003</t>
+  </si>
+  <si>
+    <t>Guru</t>
+  </si>
+  <si>
+    <t>081388990011</t>
+  </si>
+  <si>
+    <t>Ahmad Fauzi</t>
+  </si>
+  <si>
+    <t>3273021404790004</t>
+  </si>
+  <si>
+    <t>PNS</t>
   </si>
 </sst>
 </file>
@@ -97,7 +271,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xml:space="preserve">
   <numFmts count="0"/>
-  <fonts count="1">
+  <fonts count="2">
     <font>
       <b val="0"/>
       <i val="0"/>
@@ -107,16 +281,31 @@
       <color rgb="FF000000"/>
       <name val="Calibri"/>
     </font>
+    <font>
+      <b val="1"/>
+      <i val="0"/>
+      <strike val="0"/>
+      <u val="none"/>
+      <sz val="11"/>
+      <color rgb="FFFFFFFF"/>
+      <name val="Calibri"/>
+    </font>
   </fonts>
-  <fills count="2">
+  <fills count="3">
     <fill>
       <patternFill patternType="none"/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FF1E3A8A"/>
+        <bgColor rgb="FF000000"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="1">
+  <borders count="3">
     <border>
       <left/>
       <right/>
@@ -124,12 +313,48 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color rgb="FFCBD5E1"/>
+      </left>
+      <right style="thin">
+        <color rgb="FFCBD5E1"/>
+      </right>
+      <top style="thin">
+        <color rgb="FFCBD5E1"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="FFCBD5E1"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color rgb="FFE2E8F0"/>
+      </left>
+      <right style="thin">
+        <color rgb="FFE2E8F0"/>
+      </right>
+      <top style="thin">
+        <color rgb="FFE2E8F0"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="FFE2E8F0"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="1">
+  <cellXfs count="3">
     <xf xfId="0" fontId="0" numFmtId="0" fillId="0" borderId="0" applyFont="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0"/>
+    <xf xfId="0" fontId="1" numFmtId="0" fillId="2" borderId="1" applyFont="1" applyNumberFormat="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" shrinkToFit="false"/>
+    </xf>
+    <xf xfId="0" fontId="0" numFmtId="0" fillId="0" borderId="2" applyFont="0" applyNumberFormat="0" applyFill="0" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" textRotation="0" wrapText="false" shrinkToFit="false"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -429,108 +654,315 @@
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
   </sheetPr>
-  <dimension ref="A1:G4"/>
+  <dimension ref="A1:AD3"/>
   <sheetFormatPr defaultRowHeight="14.4" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col min="1" max="1" width="8.141" bestFit="true" customWidth="true" style="0"/>
     <col min="2" max="2" width="12.854" bestFit="true" customWidth="true" style="0"/>
-    <col min="3" max="3" width="15.282" bestFit="true" customWidth="true" style="0"/>
-    <col min="4" max="4" width="15.282" bestFit="true" customWidth="true" style="0"/>
-    <col min="5" max="5" width="51.845" bestFit="true" customWidth="true" style="0"/>
-    <col min="6" max="6" width="12.854" bestFit="true" customWidth="true" style="0"/>
-    <col min="7" max="7" width="12.854" bestFit="true" customWidth="true" style="0"/>
+    <col min="3" max="3" width="17.567" bestFit="true" customWidth="true" style="0"/>
+    <col min="4" max="4" width="18.71" bestFit="true" customWidth="true" style="0"/>
+    <col min="5" max="5" width="17.567" bestFit="true" customWidth="true" style="0"/>
+    <col min="6" max="6" width="51.845" bestFit="true" customWidth="true" style="0"/>
+    <col min="7" max="7" width="15.139" bestFit="true" customWidth="true" style="0"/>
+    <col min="8" max="8" width="15.139" bestFit="true" customWidth="true" style="0"/>
+    <col min="9" max="9" width="15.139" bestFit="true" customWidth="true" style="0"/>
+    <col min="10" max="10" width="13.997" bestFit="true" customWidth="true" style="0"/>
+    <col min="11" max="11" width="9.283" bestFit="true" customWidth="true" style="0"/>
+    <col min="12" max="12" width="15.282" bestFit="true" customWidth="true" style="0"/>
+    <col min="13" max="13" width="25.851" bestFit="true" customWidth="true" style="0"/>
+    <col min="14" max="14" width="26.993" bestFit="true" customWidth="true" style="0"/>
+    <col min="15" max="15" width="5.713" bestFit="true" customWidth="true" style="0"/>
+    <col min="16" max="16" width="5.713" bestFit="true" customWidth="true" style="0"/>
+    <col min="17" max="17" width="11.711" bestFit="true" customWidth="true" style="0"/>
+    <col min="18" max="18" width="16.425" bestFit="true" customWidth="true" style="0"/>
+    <col min="19" max="19" width="15.282" bestFit="true" customWidth="true" style="0"/>
+    <col min="20" max="20" width="12.854" bestFit="true" customWidth="true" style="0"/>
+    <col min="21" max="21" width="15.282" bestFit="true" customWidth="true" style="0"/>
+    <col min="22" max="22" width="15.282" bestFit="true" customWidth="true" style="0"/>
+    <col min="23" max="23" width="19.995" bestFit="true" customWidth="true" style="0"/>
+    <col min="24" max="24" width="18.71" bestFit="true" customWidth="true" style="0"/>
+    <col min="25" max="25" width="15.282" bestFit="true" customWidth="true" style="0"/>
+    <col min="26" max="26" width="13.997" bestFit="true" customWidth="true" style="0"/>
+    <col min="27" max="27" width="19.995" bestFit="true" customWidth="true" style="0"/>
+    <col min="28" max="28" width="19.852" bestFit="true" customWidth="true" style="0"/>
+    <col min="29" max="29" width="15.139" bestFit="true" customWidth="true" style="0"/>
+    <col min="30" max="30" width="13.997" bestFit="true" customWidth="true" style="0"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:7">
-      <c r="A1" t="s">
+    <row r="1" spans="1:30" customHeight="1" ht="28">
+      <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
-      <c r="B1" t="s">
+      <c r="B1" s="1" t="s">
         <v>1</v>
       </c>
-      <c r="C1" t="s">
+      <c r="C1" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="D1" t="s">
+      <c r="D1" s="1" t="s">
         <v>3</v>
       </c>
-      <c r="E1" t="s">
+      <c r="E1" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="F1" t="s">
+      <c r="F1" s="1" t="s">
         <v>5</v>
       </c>
-      <c r="G1" t="s">
+      <c r="G1" s="1" t="s">
         <v>6</v>
       </c>
+      <c r="H1" s="1" t="s">
+        <v>7</v>
+      </c>
+      <c r="I1" s="1" t="s">
+        <v>8</v>
+      </c>
+      <c r="J1" s="1" t="s">
+        <v>9</v>
+      </c>
+      <c r="K1" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="L1" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="M1" s="1" t="s">
+        <v>12</v>
+      </c>
+      <c r="N1" s="1" t="s">
+        <v>13</v>
+      </c>
+      <c r="O1" s="1" t="s">
+        <v>14</v>
+      </c>
+      <c r="P1" s="1" t="s">
+        <v>15</v>
+      </c>
+      <c r="Q1" s="1" t="s">
+        <v>16</v>
+      </c>
+      <c r="R1" s="1" t="s">
+        <v>17</v>
+      </c>
+      <c r="S1" s="1" t="s">
+        <v>18</v>
+      </c>
+      <c r="T1" s="1" t="s">
+        <v>19</v>
+      </c>
+      <c r="U1" s="1" t="s">
+        <v>20</v>
+      </c>
+      <c r="V1" s="1" t="s">
+        <v>21</v>
+      </c>
+      <c r="W1" s="1" t="s">
+        <v>22</v>
+      </c>
+      <c r="X1" s="1" t="s">
+        <v>23</v>
+      </c>
+      <c r="Y1" s="1" t="s">
+        <v>24</v>
+      </c>
+      <c r="Z1" s="1" t="s">
+        <v>25</v>
+      </c>
+      <c r="AA1" s="1" t="s">
+        <v>26</v>
+      </c>
+      <c r="AB1" s="1" t="s">
+        <v>27</v>
+      </c>
+      <c r="AC1" s="1" t="s">
+        <v>28</v>
+      </c>
+      <c r="AD1" s="1" t="s">
+        <v>29</v>
+      </c>
     </row>
-    <row r="2" spans="1:7">
-      <c r="A2">
-        <v>233001</v>
-      </c>
-      <c r="B2" t="s">
-        <v>7</v>
-      </c>
-      <c r="C2" t="s">
-        <v>8</v>
-      </c>
-      <c r="D2" t="s">
-        <v>9</v>
-      </c>
-      <c r="E2" t="s">
-        <v>10</v>
-      </c>
-      <c r="F2" t="s">
-        <v>11</v>
-      </c>
-      <c r="G2" t="s">
-        <v>12</v>
+    <row r="2" spans="1:30" customHeight="1" ht="22">
+      <c r="A2" s="2" t="s">
+        <v>30</v>
+      </c>
+      <c r="B2" s="2" t="s">
+        <v>31</v>
+      </c>
+      <c r="C2" s="2" t="s">
+        <v>32</v>
+      </c>
+      <c r="D2" s="2" t="s">
+        <v>33</v>
+      </c>
+      <c r="E2" s="2" t="s">
+        <v>34</v>
+      </c>
+      <c r="F2" s="2" t="s">
+        <v>35</v>
+      </c>
+      <c r="G2" s="2" t="s">
+        <v>36</v>
+      </c>
+      <c r="H2" s="2" t="s">
+        <v>37</v>
+      </c>
+      <c r="I2" s="2" t="s">
+        <v>38</v>
+      </c>
+      <c r="J2" s="2" t="s">
+        <v>39</v>
+      </c>
+      <c r="K2" s="2" t="s">
+        <v>40</v>
+      </c>
+      <c r="L2" s="2" t="s">
+        <v>41</v>
+      </c>
+      <c r="M2" s="2" t="s">
+        <v>42</v>
+      </c>
+      <c r="N2" s="2" t="s">
+        <v>43</v>
+      </c>
+      <c r="O2" s="2" t="s">
+        <v>44</v>
+      </c>
+      <c r="P2" s="2" t="s">
+        <v>45</v>
+      </c>
+      <c r="Q2" s="2" t="s">
+        <v>46</v>
+      </c>
+      <c r="R2" s="2" t="s">
+        <v>47</v>
+      </c>
+      <c r="S2" s="2" t="s">
+        <v>48</v>
+      </c>
+      <c r="T2" s="2" t="s">
+        <v>49</v>
+      </c>
+      <c r="U2" s="2" t="s">
+        <v>50</v>
+      </c>
+      <c r="V2" s="2" t="s">
+        <v>51</v>
+      </c>
+      <c r="W2" s="2" t="s">
+        <v>52</v>
+      </c>
+      <c r="X2" s="2" t="s">
+        <v>53</v>
+      </c>
+      <c r="Y2" s="2" t="s">
+        <v>54</v>
+      </c>
+      <c r="Z2" s="2" t="s">
+        <v>55</v>
+      </c>
+      <c r="AA2" s="2" t="s">
+        <v>56</v>
+      </c>
+      <c r="AB2" s="2" t="s">
+        <v>57</v>
+      </c>
+      <c r="AC2" s="2" t="s">
+        <v>58</v>
+      </c>
+      <c r="AD2" s="2" t="s">
+        <v>58</v>
       </c>
     </row>
-    <row r="3" spans="1:7">
-      <c r="A3">
-        <v>233002</v>
-      </c>
-      <c r="B3" t="s">
-        <v>13</v>
-      </c>
-      <c r="C3" t="s">
-        <v>14</v>
-      </c>
-      <c r="D3" t="s">
-        <v>15</v>
-      </c>
-      <c r="E3" t="s">
-        <v>16</v>
-      </c>
-      <c r="F3" t="s">
-        <v>17</v>
-      </c>
-      <c r="G3" t="s">
-        <v>18</v>
-      </c>
-    </row>
-    <row r="4" spans="1:7">
-      <c r="A4">
-        <v>233003</v>
-      </c>
-      <c r="B4" t="s">
-        <v>19</v>
-      </c>
-      <c r="C4" t="s">
-        <v>20</v>
-      </c>
-      <c r="D4" t="s">
-        <v>21</v>
-      </c>
-      <c r="E4" t="s">
-        <v>22</v>
-      </c>
-      <c r="F4" t="s">
-        <v>23</v>
-      </c>
-      <c r="G4" t="s">
-        <v>24</v>
+    <row r="3" spans="1:30" customHeight="1" ht="22">
+      <c r="A3" s="2" t="s">
+        <v>59</v>
+      </c>
+      <c r="B3" s="2" t="s">
+        <v>60</v>
+      </c>
+      <c r="C3" s="2" t="s">
+        <v>61</v>
+      </c>
+      <c r="D3" s="2" t="s">
+        <v>62</v>
+      </c>
+      <c r="E3" s="2" t="s">
+        <v>63</v>
+      </c>
+      <c r="F3" s="2" t="s">
+        <v>64</v>
+      </c>
+      <c r="G3" s="2" t="s">
+        <v>36</v>
+      </c>
+      <c r="H3" s="2" t="s">
+        <v>65</v>
+      </c>
+      <c r="I3" s="2" t="s">
+        <v>66</v>
+      </c>
+      <c r="J3" s="2" t="s">
+        <v>67</v>
+      </c>
+      <c r="K3" s="2" t="s">
+        <v>40</v>
+      </c>
+      <c r="L3" s="2" t="s">
+        <v>68</v>
+      </c>
+      <c r="M3" s="2" t="s">
+        <v>69</v>
+      </c>
+      <c r="N3" s="2" t="s">
+        <v>70</v>
+      </c>
+      <c r="O3" s="2" t="s">
+        <v>71</v>
+      </c>
+      <c r="P3" s="2" t="s">
+        <v>72</v>
+      </c>
+      <c r="Q3" s="2" t="s">
+        <v>73</v>
+      </c>
+      <c r="R3" s="2" t="s">
+        <v>74</v>
+      </c>
+      <c r="S3" s="2" t="s">
+        <v>48</v>
+      </c>
+      <c r="T3" s="2" t="s">
+        <v>49</v>
+      </c>
+      <c r="U3" s="2" t="s">
+        <v>75</v>
+      </c>
+      <c r="V3" s="2" t="s">
+        <v>76</v>
+      </c>
+      <c r="W3" s="2" t="s">
+        <v>77</v>
+      </c>
+      <c r="X3" s="2" t="s">
+        <v>78</v>
+      </c>
+      <c r="Y3" s="2" t="s">
+        <v>79</v>
+      </c>
+      <c r="Z3" s="2" t="s">
+        <v>80</v>
+      </c>
+      <c r="AA3" s="2" t="s">
+        <v>81</v>
+      </c>
+      <c r="AB3" s="2" t="s">
+        <v>82</v>
+      </c>
+      <c r="AC3" s="2" t="s">
+        <v>58</v>
+      </c>
+      <c r="AD3" s="2" t="s">
+        <v>58</v>
       </c>
     </row>
   </sheetData>

</xml_diff>